<commit_message>
made some new models and edited other ones to allow for more analysis of absorption data.
</commit_message>
<xml_diff>
--- a/Data/AFRL Compiled EA Data/K-values.xlsx
+++ b/Data/AFRL Compiled EA Data/K-values.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byu-my.sharepoint.com/personal/carterms_byu_edu/Documents/Documents/Research/Spectra-Link/Data/AFRL Compiled EA Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{6F16E2B4-E4C3-470E-B7B2-B88B7885A5D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21E119A2-E931-45D9-B2BF-69EC53834367}"/>
+  <xr:revisionPtr revIDLastSave="191" documentId="8_{6F16E2B4-E4C3-470E-B7B2-B88B7885A5D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{032ABBE4-58CF-4591-A20C-7FA09C0BFE05}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CD00ED08-05B2-419B-B8E3-F14F394DB09C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{CD00ED08-05B2-419B-B8E3-F14F394DB09C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="16">
   <si>
     <t>16K</t>
   </si>
@@ -72,12 +73,30 @@
   </si>
   <si>
     <t>Range 5</t>
+  </si>
+  <si>
+    <t>uncert</t>
+  </si>
+  <si>
+    <t>left</t>
+  </si>
+  <si>
+    <t>right</t>
+  </si>
+  <si>
+    <t>diff</t>
+  </si>
+  <si>
+    <t>less than 20 meV can't distinguish well</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -113,8 +132,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -130,6 +151,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -449,109 +474,656 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0012194-FA2B-46ED-977F-334407AD58A2}">
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3">
-        <v>1.7370000000000001</v>
-      </c>
-      <c r="C3">
-        <v>1.736</v>
-      </c>
-      <c r="D3">
-        <v>1.889</v>
-      </c>
-      <c r="E3">
-        <v>1.883</v>
-      </c>
-      <c r="F3">
-        <v>1.851</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="2">
+        <v>1.6659999999999999</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.03</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1.65</v>
+      </c>
+      <c r="E3" s="2">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1.669</v>
+      </c>
+      <c r="G3" s="2">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1.702</v>
+      </c>
+      <c r="I3" s="2">
+        <v>4.5999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1.9119999999999999</v>
-      </c>
-      <c r="C4">
-        <v>1.7150000000000001</v>
-      </c>
-      <c r="D4">
-        <v>1.7310000000000001</v>
-      </c>
-      <c r="E4">
-        <v>1.748</v>
-      </c>
-      <c r="F4">
-        <v>1.8160000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="2">
+        <v>1.915</v>
+      </c>
+      <c r="C4" s="2">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1.831</v>
+      </c>
+      <c r="E4" s="2">
+        <v>9.1999999999999998E-2</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1.736</v>
+      </c>
+      <c r="G4" s="2">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="H4" s="2">
+        <v>1.742</v>
+      </c>
+      <c r="I4" s="2">
+        <v>2.9000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5">
-        <v>1.9079999999999999</v>
-      </c>
-      <c r="C5">
-        <v>1.9279999999999999</v>
-      </c>
-      <c r="D5">
-        <v>1.641</v>
-      </c>
-      <c r="E5">
-        <v>1.736</v>
-      </c>
-      <c r="F5">
-        <v>1.8340000000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="2">
+        <v>1.79</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1.9530000000000001</v>
+      </c>
+      <c r="E5" s="2">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1.524</v>
+      </c>
+      <c r="G5" s="2">
+        <v>4.2999999999999997E-2</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1.663</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>2.72</v>
-      </c>
-      <c r="C6">
-        <v>1.5940000000000001</v>
-      </c>
-      <c r="D6">
-        <v>1.877</v>
-      </c>
-      <c r="E6">
-        <v>1.9079999999999999</v>
-      </c>
-      <c r="F6">
-        <v>1.919</v>
+      <c r="B6" s="2">
+        <v>2.31</v>
+      </c>
+      <c r="C6" s="2">
+        <v>4.2999999999999997E-2</v>
+      </c>
+      <c r="D6" s="2">
+        <v>2.6459999999999999</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0.66200000000000003</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1.833</v>
+      </c>
+      <c r="G6" s="2">
+        <v>2.7E-2</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1.897</v>
+      </c>
+      <c r="I6" s="2">
+        <v>2.8000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H10" t="s">
+        <v>9</v>
+      </c>
+      <c r="I10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1.67</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1.65</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1.67</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0.06</v>
+      </c>
+      <c r="H11" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="I11" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="K11">
+        <v>1.6659999999999999</v>
+      </c>
+      <c r="L11">
+        <v>0.03</v>
+      </c>
+      <c r="M11">
+        <v>1.65</v>
+      </c>
+      <c r="N11">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="O11">
+        <v>1.669</v>
+      </c>
+      <c r="P11">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="Q11">
+        <v>1.702</v>
+      </c>
+      <c r="R11">
+        <v>4.5999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="1">
+        <v>1.92</v>
+      </c>
+      <c r="C12" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1.83</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.09</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1.74</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="H12" s="1">
+        <v>1.74</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="K12">
+        <v>1.915</v>
+      </c>
+      <c r="L12">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="M12">
+        <v>1.831</v>
+      </c>
+      <c r="N12">
+        <v>9.1999999999999998E-2</v>
+      </c>
+      <c r="O12">
+        <v>1.736</v>
+      </c>
+      <c r="P12">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="Q12">
+        <v>1.742</v>
+      </c>
+      <c r="R12">
+        <v>2.9000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="1">
+        <v>1.79</v>
+      </c>
+      <c r="C13" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1.95</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="F13" s="1">
+        <v>1.52</v>
+      </c>
+      <c r="G13" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="H13" s="1">
+        <v>1.66</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="K13">
+        <v>1.79</v>
+      </c>
+      <c r="L13">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="M13">
+        <v>1.9530000000000001</v>
+      </c>
+      <c r="N13">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="O13">
+        <v>1.524</v>
+      </c>
+      <c r="P13">
+        <v>4.2999999999999997E-2</v>
+      </c>
+      <c r="Q13">
+        <v>1.663</v>
+      </c>
+      <c r="R13">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="1">
+        <v>2.31</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="D14" s="1">
+        <v>2.65</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0.66</v>
+      </c>
+      <c r="F14" s="1">
+        <v>1.83</v>
+      </c>
+      <c r="G14" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="H14" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="I14" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="K14">
+        <v>2.31</v>
+      </c>
+      <c r="L14">
+        <v>4.2999999999999997E-2</v>
+      </c>
+      <c r="M14">
+        <v>2.6459999999999999</v>
+      </c>
+      <c r="N14">
+        <v>0.66200000000000003</v>
+      </c>
+      <c r="O14">
+        <v>1.833</v>
+      </c>
+      <c r="P14">
+        <v>2.7E-2</v>
+      </c>
+      <c r="Q14">
+        <v>1.897</v>
+      </c>
+      <c r="R14">
+        <v>2.8000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" t="s">
+        <v>14</v>
+      </c>
+      <c r="K17" t="s">
+        <v>12</v>
+      </c>
+      <c r="L17" t="s">
+        <v>13</v>
+      </c>
+      <c r="M17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" t="str">
+        <f>"a = " &amp; B11 &amp; " ± " &amp; C11</f>
+        <v>a = 1.67 ± 0.03</v>
+      </c>
+      <c r="C18" t="str">
+        <f>"a = " &amp; B12 &amp; " ± " &amp; C12</f>
+        <v>a = 1.92 ± 0.05</v>
+      </c>
+      <c r="E18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F18">
+        <v>2.5529999999999999</v>
+      </c>
+      <c r="G18">
+        <v>2.5819999999999999</v>
+      </c>
+      <c r="H18">
+        <f>G18-F18</f>
+        <v>2.8999999999999915E-2</v>
+      </c>
+      <c r="J18" t="s">
+        <v>4</v>
+      </c>
+      <c r="K18">
+        <v>2.5630000000000002</v>
+      </c>
+      <c r="L18">
+        <v>2.5859999999999999</v>
+      </c>
+      <c r="M18">
+        <f>L18-K18</f>
+        <v>2.2999999999999687E-2</v>
+      </c>
+      <c r="N18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="str">
+        <f>"b = " &amp; D11 &amp; " ± " &amp; E11</f>
+        <v>b = 1.65 ± 0.03</v>
+      </c>
+      <c r="C19" t="str">
+        <f>"b = " &amp; D12 &amp; " ± " &amp; E12</f>
+        <v>b = 1.83 ± 0.09</v>
+      </c>
+      <c r="E19" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19">
+        <v>2.5449999999999999</v>
+      </c>
+      <c r="G19">
+        <v>2.5960000000000001</v>
+      </c>
+      <c r="H19">
+        <f t="shared" ref="H19:H21" si="0">G19-F19</f>
+        <v>5.1000000000000156E-2</v>
+      </c>
+      <c r="J19" t="s">
+        <v>3</v>
+      </c>
+      <c r="K19">
+        <v>2.556</v>
+      </c>
+      <c r="L19">
+        <v>2.5790000000000002</v>
+      </c>
+      <c r="M19">
+        <f t="shared" ref="M19:M21" si="1">L19-K19</f>
+        <v>2.3000000000000131E-2</v>
+      </c>
+      <c r="O19">
+        <f t="shared" ref="O19:O20" si="2">M19-H19</f>
+        <v>-2.8000000000000025E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" t="str">
+        <f>"c = " &amp; F11 &amp; " ± " &amp; G11</f>
+        <v>c = 1.67 ± 0.06</v>
+      </c>
+      <c r="C20" t="str">
+        <f>"c = " &amp; F12 &amp; " ± " &amp; G12</f>
+        <v>c = 1.74 ± 0.04</v>
+      </c>
+      <c r="E20" t="s">
+        <v>2</v>
+      </c>
+      <c r="F20">
+        <v>2.536</v>
+      </c>
+      <c r="G20">
+        <v>2.5910000000000002</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="0"/>
+        <v>5.500000000000016E-2</v>
+      </c>
+      <c r="J20" t="s">
+        <v>2</v>
+      </c>
+      <c r="K20">
+        <v>2.5449999999999999</v>
+      </c>
+      <c r="L20">
+        <v>2.5739999999999998</v>
+      </c>
+      <c r="M20">
+        <f t="shared" si="1"/>
+        <v>2.8999999999999915E-2</v>
+      </c>
+      <c r="O20">
+        <f t="shared" si="2"/>
+        <v>-2.6000000000000245E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" t="str">
+        <f>"d = " &amp; H11 &amp; "0 ± " &amp; I11</f>
+        <v>d = 1.70 ± 0.05</v>
+      </c>
+      <c r="C21" t="str">
+        <f>"d = " &amp; H12 &amp; " ± " &amp; I12</f>
+        <v>d = 1.74 ± 0.03</v>
+      </c>
+      <c r="E21" t="s">
+        <v>5</v>
+      </c>
+      <c r="F21">
+        <v>2.556</v>
+      </c>
+      <c r="G21">
+        <v>2.6190000000000002</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="0"/>
+        <v>6.3000000000000167E-2</v>
+      </c>
+      <c r="J21" t="s">
+        <v>5</v>
+      </c>
+      <c r="K21">
+        <v>2.5659999999999998</v>
+      </c>
+      <c r="L21">
+        <v>2.6059999999999999</v>
+      </c>
+      <c r="M21">
+        <f t="shared" si="1"/>
+        <v>4.0000000000000036E-2</v>
+      </c>
+      <c r="O21">
+        <f>M21-H21</f>
+        <v>-2.3000000000000131E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="str">
+        <f>"a = " &amp; B14 &amp; " ± " &amp; C14</f>
+        <v>a = 2.31 ± 0.04</v>
+      </c>
+      <c r="C22" t="str">
+        <f>"a = " &amp; B13 &amp; " ± " &amp; C13 &amp; "0"</f>
+        <v>a = 1.79 ± 0.10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="str">
+        <f>"b = " &amp; D14 &amp; " ± " &amp; E14</f>
+        <v>b = 2.65 ± 0.66</v>
+      </c>
+      <c r="C23" t="str">
+        <f>"b = " &amp; D13 &amp; " ± " &amp; E13</f>
+        <v>b = 1.95 ± 0.04</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="str">
+        <f>"c = " &amp; F14 &amp; " ± " &amp; G14</f>
+        <v>c = 1.83 ± 0.03</v>
+      </c>
+      <c r="C24" t="str">
+        <f>"c = " &amp; F13 &amp; " ± " &amp; G13</f>
+        <v>c = 1.52 ± 0.04</v>
+      </c>
+      <c r="F24">
+        <f>K18-F18</f>
+        <v>1.0000000000000231E-2</v>
+      </c>
+      <c r="G24">
+        <f>L18-G18</f>
+        <v>4.0000000000000036E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="str">
+        <f>"d = " &amp; H14 &amp; "0 ± " &amp; I14</f>
+        <v>d = 1.90 ± 0.03</v>
+      </c>
+      <c r="C25" t="str">
+        <f>"d = " &amp; H13 &amp; " ± " &amp; I13</f>
+        <v>d = 1.66 ± 0.04</v>
+      </c>
+      <c r="F25">
+        <f t="shared" ref="F25:G25" si="3">K19-F19</f>
+        <v>1.1000000000000121E-2</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="3"/>
+        <v>-1.6999999999999904E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F26">
+        <f t="shared" ref="F26:G26" si="4">K20-F20</f>
+        <v>8.999999999999897E-3</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="4"/>
+        <v>-1.7000000000000348E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F27">
+        <f t="shared" ref="F27:G27" si="5">K21-F21</f>
+        <v>9.9999999999997868E-3</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="5"/>
+        <v>-1.3000000000000345E-2</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -599,5 +1171,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>